<commit_message>
Add: alteração de datas
</commit_message>
<xml_diff>
--- a/inputs/Gerenciamento de Projetos .xlsx
+++ b/inputs/Gerenciamento de Projetos .xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupochibatao-my.sharepoint.com/personal/artur_almeida_grupochibatao_com_br/Documents/Documentos/progs/PowerBI_Projetos/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_4F87750511974F703C528916B4EB3D35546076DB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E0B28BC-3A3B-4CFA-9F6E-DB9A4B070E15}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_4F87750511974F703C028F59380B3D355460713C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36561063-090D-41FC-972B-DA62AFB8C588}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tarefas" sheetId="1" r:id="rId1"/>
     <sheet name="Nome do plano" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tarefas!$C$1:$C$75</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -77,45 +80,57 @@
     <t>Descrição</t>
   </si>
   <si>
+    <t>yVYhkEPnrkGIoTpyuQGT4WUAFGJw</t>
+  </si>
+  <si>
+    <t>Cancelamento de entrada - Projeto de suporte</t>
+  </si>
+  <si>
+    <t>Execução</t>
+  </si>
+  <si>
+    <t>Não iniciado</t>
+  </si>
+  <si>
+    <t>Importante</t>
+  </si>
+  <si>
+    <t>Michael Oneil;Artur Almeida</t>
+  </si>
+  <si>
+    <t>Artur Almeida</t>
+  </si>
+  <si>
+    <t>09/07/2025</t>
+  </si>
+  <si>
+    <t>08/07/2025</t>
+  </si>
+  <si>
+    <t>11/07/2025</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Alta Prioridade</t>
+  </si>
+  <si>
     <t>33xcpcqGakCDcbja5yzfLGUADDlp</t>
   </si>
   <si>
     <t>Novo PortPlanner</t>
   </si>
   <si>
-    <t>Execução</t>
-  </si>
-  <si>
-    <t>Não iniciado</t>
-  </si>
-  <si>
-    <t>Importante</t>
-  </si>
-  <si>
-    <t>Michael Oneil;Artur Almeida</t>
-  </si>
-  <si>
-    <t>Artur Almeida</t>
-  </si>
-  <si>
-    <t>08/07/2025</t>
-  </si>
-  <si>
     <t>01/05/2024</t>
   </si>
   <si>
     <t>31/07/2025</t>
   </si>
   <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Alta Prioridade</t>
-  </si>
-  <si>
     <t>frfoHWQbrE2rkF_Yib7tBWUALtn-</t>
   </si>
   <si>
@@ -206,9 +221,6 @@
     <t>04/07/2025</t>
   </si>
   <si>
-    <t>11/07/2025</t>
-  </si>
-  <si>
     <t>URGENTE</t>
   </si>
   <si>
@@ -221,27 +233,6 @@
     <t>03/07/2025</t>
   </si>
   <si>
-    <t>tZxKh7EDgkO30JTpIZGtMWUAGIHw</t>
-  </si>
-  <si>
-    <t>Relatorio de unidades no canal verde do entreposto - Geração de relatório via script</t>
-  </si>
-  <si>
-    <t>Concluidas</t>
-  </si>
-  <si>
-    <t>Concluída</t>
-  </si>
-  <si>
-    <t>02/07/2025</t>
-  </si>
-  <si>
-    <t>09/07/2025</t>
-  </si>
-  <si>
-    <t>Solicitado pela diretoria</t>
-  </si>
-  <si>
     <t>TJ989zRAsECgZj29xMZIu2UAC_xU</t>
   </si>
   <si>
@@ -254,7 +245,7 @@
     <t>DwrBACgLSU2oTbRQjENr_2UAB7nP</t>
   </si>
   <si>
-    <t>segundo teste do checklist-guindaste</t>
+    <t>Segundo teste do checklist-guindaste</t>
   </si>
   <si>
     <t>Aguardando validação</t>
@@ -344,9 +335,9 @@
     <t>10/06/2025</t>
   </si>
   <si>
-    <t>**Descrição do teste realizado em 10/06/2025:**_x000D_
+    <t>Descrição do teste realizado em 10/06/2025:_x000D_
 _x000D_
-Foi realizada uma alteração no processo para capturar o código da avaria automaticamente, eliminando a necessidade de digitar manualmente o nome da avaria. Além disso, a opção de informar o lacre será removida.</t>
+Foi realizada uma alteração no processo para capturar o código da avaria automaticamente, eliminando a necessidade de digitar manualmente o nome da avaria. Além disso, a opção de informar o lacre será removida</t>
   </si>
   <si>
     <t>dXkqgRgCbkSg9CZd49KpNmUALk29</t>
@@ -553,6 +544,9 @@
   </si>
   <si>
     <t>Atualização da Plataforma do Launcher ModallWeb</t>
+  </si>
+  <si>
+    <t>Baixa Prioridade;Sem Previsão</t>
   </si>
   <si>
     <t>Sem previsão</t>
@@ -613,6 +607,24 @@
 Dividir em grupos catracas de refeitório de catracas de entrada e saída.</t>
   </si>
   <si>
+    <t>tZxKh7EDgkO30JTpIZGtMWUAGIHw</t>
+  </si>
+  <si>
+    <t>Relatorio de unidades no canal verde do entreposto - Geração de relatório via script</t>
+  </si>
+  <si>
+    <t>Concluidas</t>
+  </si>
+  <si>
+    <t>Concluída</t>
+  </si>
+  <si>
+    <t>02/07/2025</t>
+  </si>
+  <si>
+    <t>Solicitado pela diretoria</t>
+  </si>
+  <si>
     <t>p789wN0uJUCC5t7nI2sSjGUAHsnn</t>
   </si>
   <si>
@@ -646,9 +658,6 @@
     <t>Corrigir Consulta da Unidade - DEPOT</t>
   </si>
   <si>
-    <t>Artur Almeida;Michael Oneil</t>
-  </si>
-  <si>
     <t>zKkRumS_kEaTUBAB1hskk2UAFf5I</t>
   </si>
   <si>
@@ -758,12 +767,6 @@
   </si>
   <si>
     <t>Checklist de empilhadeira MODALLCHECK Remoção</t>
-  </si>
-  <si>
-    <t>yVYhkEPnrkGIoTpyuQGT4WUAFGJw</t>
-  </si>
-  <si>
-    <t>Cancelamento de entrada - Projeto de suporte</t>
   </si>
   <si>
     <t>Nome do plano</t>
@@ -1155,6 +1158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R75"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1305,13 +1309,13 @@
         <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="J3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
         <v>28</v>
@@ -1337,10 +1341,10 @@
     </row>
     <row r="4" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
         <v>20</v>
@@ -1358,13 +1362,13 @@
         <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I4" t="s">
         <v>29</v>
       </c>
       <c r="J4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K4" t="s">
         <v>28</v>
@@ -1390,10 +1394,10 @@
     </row>
     <row r="5" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -1411,13 +1415,13 @@
         <v>24</v>
       </c>
       <c r="H5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J5" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="K5" t="s">
         <v>28</v>
@@ -1439,9 +1443,6 @@
       </c>
       <c r="Q5" t="s">
         <v>30</v>
-      </c>
-      <c r="R5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
@@ -1467,13 +1468,13 @@
         <v>24</v>
       </c>
       <c r="H6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="J6" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="K6" t="s">
         <v>28</v>
@@ -1497,18 +1498,18 @@
         <v>30</v>
       </c>
       <c r="R6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
         <v>21</v>
@@ -1523,13 +1524,13 @@
         <v>24</v>
       </c>
       <c r="H7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I7" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="J7" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="K7" t="s">
         <v>28</v>
@@ -1552,22 +1553,25 @@
       <c r="Q7" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="R7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F8" t="s">
         <v>23</v>
@@ -1576,7 +1580,7 @@
         <v>24</v>
       </c>
       <c r="H8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I8" t="s">
         <v>29</v>
@@ -1603,10 +1607,10 @@
         <v>29</v>
       </c>
       <c r="Q8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -1614,13 +1618,13 @@
         <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="F9" t="s">
         <v>23</v>
@@ -1629,7 +1633,7 @@
         <v>24</v>
       </c>
       <c r="H9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I9" t="s">
         <v>29</v>
@@ -1656,24 +1660,24 @@
         <v>29</v>
       </c>
       <c r="Q9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F10" t="s">
         <v>23</v>
@@ -1682,7 +1686,7 @@
         <v>24</v>
       </c>
       <c r="H10" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="I10" t="s">
         <v>29</v>
@@ -1709,24 +1713,24 @@
         <v>29</v>
       </c>
       <c r="Q10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" t="s">
         <v>56</v>
-      </c>
-      <c r="C11" t="s">
-        <v>52</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="F11" t="s">
         <v>23</v>
@@ -1735,7 +1739,7 @@
         <v>24</v>
       </c>
       <c r="H11" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="I11" t="s">
         <v>29</v>
@@ -1762,24 +1766,24 @@
         <v>29</v>
       </c>
       <c r="Q11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="F12" t="s">
         <v>23</v>
@@ -1788,13 +1792,13 @@
         <v>24</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="I12" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="J12" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="K12" t="s">
         <v>28</v>
@@ -1815,24 +1819,24 @@
         <v>29</v>
       </c>
       <c r="Q12" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="F13" t="s">
         <v>23</v>
@@ -1841,37 +1845,37 @@
         <v>24</v>
       </c>
       <c r="H13" t="s">
+        <v>64</v>
+      </c>
+      <c r="I13" t="s">
+        <v>43</v>
+      </c>
+      <c r="J13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" t="s">
+        <v>28</v>
+      </c>
+      <c r="L13" t="s">
+        <v>28</v>
+      </c>
+      <c r="M13" t="s">
+        <v>29</v>
+      </c>
+      <c r="N13" t="s">
+        <v>29</v>
+      </c>
+      <c r="O13" t="s">
+        <v>29</v>
+      </c>
+      <c r="P13" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q13" t="s">
         <v>65</v>
       </c>
-      <c r="I13" t="s">
-        <v>29</v>
-      </c>
-      <c r="J13" t="s">
-        <v>29</v>
-      </c>
-      <c r="K13" t="s">
-        <v>28</v>
-      </c>
-      <c r="L13" t="s">
-        <v>28</v>
-      </c>
-      <c r="M13" t="s">
-        <v>29</v>
-      </c>
-      <c r="N13" t="s">
-        <v>29</v>
-      </c>
-      <c r="O13" t="s">
-        <v>29</v>
-      </c>
-      <c r="P13" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>66</v>
       </c>
@@ -1879,69 +1883,66 @@
         <v>67</v>
       </c>
       <c r="C14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" t="s">
         <v>68</v>
       </c>
-      <c r="D14" t="s">
+      <c r="I14" t="s">
+        <v>29</v>
+      </c>
+      <c r="J14" t="s">
+        <v>29</v>
+      </c>
+      <c r="K14" t="s">
+        <v>28</v>
+      </c>
+      <c r="L14" t="s">
+        <v>28</v>
+      </c>
+      <c r="M14" t="s">
+        <v>29</v>
+      </c>
+      <c r="N14" t="s">
+        <v>29</v>
+      </c>
+      <c r="O14" t="s">
+        <v>29</v>
+      </c>
+      <c r="P14" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>69</v>
       </c>
-      <c r="E14" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" t="s">
-        <v>23</v>
-      </c>
-      <c r="G14" t="s">
-        <v>24</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="B15" t="s">
         <v>70</v>
       </c>
-      <c r="I14" t="s">
-        <v>60</v>
-      </c>
-      <c r="J14" t="s">
-        <v>60</v>
-      </c>
-      <c r="K14" t="s">
-        <v>28</v>
-      </c>
-      <c r="L14" t="s">
-        <v>28</v>
-      </c>
-      <c r="M14" t="s">
-        <v>71</v>
-      </c>
-      <c r="N14" t="s">
-        <v>24</v>
-      </c>
-      <c r="O14" t="s">
-        <v>29</v>
-      </c>
-      <c r="P14" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>62</v>
-      </c>
-      <c r="R14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>73</v>
-      </c>
-      <c r="B15" t="s">
-        <v>74</v>
-      </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
         <v>21</v>
       </c>
       <c r="E15" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F15" t="s">
         <v>23</v>
@@ -1950,7 +1951,7 @@
         <v>24</v>
       </c>
       <c r="H15" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I15" t="s">
         <v>29</v>
@@ -1977,24 +1978,24 @@
         <v>29</v>
       </c>
       <c r="Q15" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D16" t="s">
         <v>21</v>
       </c>
       <c r="E16" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F16" t="s">
         <v>24</v>
@@ -2003,19 +2004,19 @@
         <v>24</v>
       </c>
       <c r="H16" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" t="s">
         <v>75</v>
       </c>
-      <c r="I16" t="s">
-        <v>79</v>
-      </c>
       <c r="J16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K16" t="s">
         <v>28</v>
       </c>
       <c r="L16" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="M16" t="s">
         <v>29</v>
@@ -2030,15 +2031,15 @@
         <v>29</v>
       </c>
       <c r="Q16" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
@@ -2047,7 +2048,7 @@
         <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F17" t="s">
         <v>23</v>
@@ -2056,51 +2057,51 @@
         <v>24</v>
       </c>
       <c r="H17" t="s">
+        <v>79</v>
+      </c>
+      <c r="I17" t="s">
+        <v>80</v>
+      </c>
+      <c r="J17" t="s">
+        <v>37</v>
+      </c>
+      <c r="K17" t="s">
+        <v>28</v>
+      </c>
+      <c r="L17" t="s">
+        <v>28</v>
+      </c>
+      <c r="M17" t="s">
+        <v>29</v>
+      </c>
+      <c r="N17" t="s">
+        <v>29</v>
+      </c>
+      <c r="O17" t="s">
+        <v>29</v>
+      </c>
+      <c r="P17" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" t="s">
         <v>83</v>
       </c>
-      <c r="I17" t="s">
-        <v>84</v>
-      </c>
-      <c r="J17" t="s">
-        <v>33</v>
-      </c>
-      <c r="K17" t="s">
-        <v>28</v>
-      </c>
-      <c r="L17" t="s">
-        <v>28</v>
-      </c>
-      <c r="M17" t="s">
-        <v>29</v>
-      </c>
-      <c r="N17" t="s">
-        <v>29</v>
-      </c>
-      <c r="O17" t="s">
-        <v>29</v>
-      </c>
-      <c r="P17" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>86</v>
-      </c>
-      <c r="B18" t="s">
-        <v>87</v>
-      </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D18" t="s">
         <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F18" t="s">
         <v>23</v>
@@ -2109,7 +2110,7 @@
         <v>24</v>
       </c>
       <c r="H18" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I18" t="s">
         <v>29</v>
@@ -2130,24 +2131,24 @@
         <v>29</v>
       </c>
       <c r="O18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P18" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="Q18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" t="s">
-        <v>45</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -2159,10 +2160,10 @@
         <v>23</v>
       </c>
       <c r="G19" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H19" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="I19" t="s">
         <v>29</v>
@@ -2192,18 +2193,18 @@
         <v>30</v>
       </c>
       <c r="R19" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D20" t="s">
         <v>21</v>
@@ -2218,7 +2219,7 @@
         <v>24</v>
       </c>
       <c r="H20" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="I20" t="s">
         <v>29</v>
@@ -2248,15 +2249,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B21" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D21" t="s">
         <v>21</v>
@@ -2271,7 +2272,7 @@
         <v>24</v>
       </c>
       <c r="H21" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="I21" t="s">
         <v>29</v>
@@ -2301,21 +2302,21 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D22" t="s">
         <v>21</v>
       </c>
       <c r="E22" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F22" t="s">
         <v>23</v>
@@ -2324,7 +2325,7 @@
         <v>24</v>
       </c>
       <c r="H22" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="I22" t="s">
         <v>29</v>
@@ -2351,24 +2352,24 @@
         <v>29</v>
       </c>
       <c r="Q22" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D23" t="s">
         <v>21</v>
       </c>
       <c r="E23" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F23" t="s">
         <v>23</v>
@@ -2377,7 +2378,7 @@
         <v>24</v>
       </c>
       <c r="H23" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="I23" t="s">
         <v>29</v>
@@ -2404,24 +2405,24 @@
         <v>29</v>
       </c>
       <c r="Q23" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B24" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C24" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
         <v>21</v>
       </c>
       <c r="E24" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F24" t="s">
         <v>23</v>
@@ -2430,13 +2431,13 @@
         <v>24</v>
       </c>
       <c r="H24" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="I24" t="s">
         <v>29</v>
       </c>
       <c r="J24" t="s">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="K24" t="s">
         <v>28</v>
@@ -2457,27 +2458,27 @@
         <v>29</v>
       </c>
       <c r="Q24" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="R24" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B25" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C25" t="s">
         <v>20</v>
       </c>
       <c r="D25" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E25" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F25" t="s">
         <v>24</v>
@@ -2486,13 +2487,13 @@
         <v>24</v>
       </c>
       <c r="H25" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="I25" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="J25" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="K25" t="s">
         <v>28</v>
@@ -2513,21 +2514,21 @@
         <v>29</v>
       </c>
       <c r="Q25" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B26" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C26" t="s">
         <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E26" t="s">
         <v>22</v>
@@ -2536,16 +2537,16 @@
         <v>23</v>
       </c>
       <c r="G26" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H26" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I26" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="J26" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K26" t="s">
         <v>28</v>
@@ -2569,15 +2570,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B27" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D27" t="s">
         <v>21</v>
@@ -2589,57 +2590,57 @@
         <v>29</v>
       </c>
       <c r="G27" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H27" t="s">
+        <v>112</v>
+      </c>
+      <c r="I27" t="s">
+        <v>29</v>
+      </c>
+      <c r="J27" t="s">
+        <v>29</v>
+      </c>
+      <c r="K27" t="s">
+        <v>28</v>
+      </c>
+      <c r="L27" t="s">
+        <v>28</v>
+      </c>
+      <c r="M27" t="s">
+        <v>29</v>
+      </c>
+      <c r="N27" t="s">
+        <v>29</v>
+      </c>
+      <c r="O27" t="s">
+        <v>29</v>
+      </c>
+      <c r="P27" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>53</v>
+      </c>
+      <c r="R27" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>116</v>
       </c>
-      <c r="I27" t="s">
-        <v>29</v>
-      </c>
-      <c r="J27" t="s">
-        <v>29</v>
-      </c>
-      <c r="K27" t="s">
-        <v>28</v>
-      </c>
-      <c r="L27" t="s">
-        <v>28</v>
-      </c>
-      <c r="M27" t="s">
-        <v>29</v>
-      </c>
-      <c r="N27" t="s">
-        <v>29</v>
-      </c>
-      <c r="O27" t="s">
-        <v>29</v>
-      </c>
-      <c r="P27" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q27" t="s">
-        <v>49</v>
-      </c>
-      <c r="R27" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="28" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>120</v>
-      </c>
       <c r="B28" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D28" t="s">
         <v>21</v>
       </c>
       <c r="E28" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F28" t="s">
         <v>29</v>
@@ -2648,7 +2649,7 @@
         <v>24</v>
       </c>
       <c r="H28" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I28" t="s">
         <v>29</v>
@@ -2669,30 +2670,30 @@
         <v>29</v>
       </c>
       <c r="O28" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P28" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="Q28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D29" t="s">
         <v>21</v>
       </c>
       <c r="E29" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F29" t="s">
         <v>29</v>
@@ -2701,51 +2702,51 @@
         <v>24</v>
       </c>
       <c r="H29" t="s">
+        <v>118</v>
+      </c>
+      <c r="I29" t="s">
+        <v>29</v>
+      </c>
+      <c r="J29" t="s">
+        <v>29</v>
+      </c>
+      <c r="K29" t="s">
+        <v>28</v>
+      </c>
+      <c r="L29" t="s">
+        <v>28</v>
+      </c>
+      <c r="M29" t="s">
+        <v>29</v>
+      </c>
+      <c r="N29" t="s">
+        <v>29</v>
+      </c>
+      <c r="O29" t="s">
+        <v>84</v>
+      </c>
+      <c r="P29" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>122</v>
       </c>
-      <c r="I29" t="s">
-        <v>29</v>
-      </c>
-      <c r="J29" t="s">
-        <v>29</v>
-      </c>
-      <c r="K29" t="s">
-        <v>28</v>
-      </c>
-      <c r="L29" t="s">
-        <v>28</v>
-      </c>
-      <c r="M29" t="s">
-        <v>29</v>
-      </c>
-      <c r="N29" t="s">
-        <v>29</v>
-      </c>
-      <c r="O29" t="s">
-        <v>88</v>
-      </c>
-      <c r="P29" t="s">
+      <c r="B30" t="s">
         <v>123</v>
       </c>
-      <c r="Q29" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="30" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>126</v>
-      </c>
-      <c r="B30" t="s">
-        <v>127</v>
-      </c>
       <c r="C30" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D30" t="s">
         <v>21</v>
       </c>
       <c r="E30" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F30" t="s">
         <v>23</v>
@@ -2754,7 +2755,7 @@
         <v>24</v>
       </c>
       <c r="H30" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I30" t="s">
         <v>29</v>
@@ -2781,15 +2782,15 @@
         <v>29</v>
       </c>
       <c r="Q30" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B31" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C31" t="s">
         <v>20</v>
@@ -2807,13 +2808,13 @@
         <v>24</v>
       </c>
       <c r="H31" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I31" t="s">
         <v>29</v>
       </c>
       <c r="J31" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="K31" t="s">
         <v>28</v>
@@ -2837,21 +2838,21 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D32" t="s">
         <v>21</v>
       </c>
       <c r="E32" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F32" t="s">
         <v>23</v>
@@ -2860,7 +2861,7 @@
         <v>24</v>
       </c>
       <c r="H32" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I32" t="s">
         <v>29</v>
@@ -2887,18 +2888,18 @@
         <v>29</v>
       </c>
       <c r="Q32" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B33" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D33" t="s">
         <v>21</v>
@@ -2913,7 +2914,7 @@
         <v>24</v>
       </c>
       <c r="H33" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I33" t="s">
         <v>29</v>
@@ -2934,33 +2935,33 @@
         <v>29</v>
       </c>
       <c r="O33" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P33" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="Q33" t="s">
         <v>30</v>
       </c>
       <c r="R33" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B34" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C34" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
       </c>
       <c r="E34" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F34" t="s">
         <v>23</v>
@@ -2969,7 +2970,7 @@
         <v>24</v>
       </c>
       <c r="H34" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I34" t="s">
         <v>29</v>
@@ -2996,24 +2997,24 @@
         <v>29</v>
       </c>
       <c r="Q34" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B35" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D35" t="s">
         <v>21</v>
       </c>
       <c r="E35" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F35" t="s">
         <v>23</v>
@@ -3022,7 +3023,7 @@
         <v>24</v>
       </c>
       <c r="H35" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I35" t="s">
         <v>29</v>
@@ -3049,24 +3050,24 @@
         <v>29</v>
       </c>
       <c r="Q35" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B36" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D36" t="s">
         <v>21</v>
       </c>
       <c r="E36" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F36" t="s">
         <v>23</v>
@@ -3075,7 +3076,7 @@
         <v>24</v>
       </c>
       <c r="H36" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I36" t="s">
         <v>29</v>
@@ -3102,18 +3103,18 @@
         <v>29</v>
       </c>
       <c r="Q36" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>138</v>
+      </c>
+      <c r="B37" t="s">
+        <v>139</v>
+      </c>
+      <c r="C37" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>142</v>
-      </c>
-      <c r="B37" t="s">
-        <v>143</v>
-      </c>
-      <c r="C37" t="s">
-        <v>45</v>
       </c>
       <c r="D37" t="s">
         <v>21</v>
@@ -3128,7 +3129,7 @@
         <v>24</v>
       </c>
       <c r="H37" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I37" t="s">
         <v>29</v>
@@ -3158,21 +3159,21 @@
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B38" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C38" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D38" t="s">
         <v>21</v>
       </c>
       <c r="E38" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F38" t="s">
         <v>23</v>
@@ -3181,7 +3182,7 @@
         <v>24</v>
       </c>
       <c r="H38" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I38" t="s">
         <v>29</v>
@@ -3208,18 +3209,18 @@
         <v>29</v>
       </c>
       <c r="Q38" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B39" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C39" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D39" t="s">
         <v>21</v>
@@ -3234,7 +3235,7 @@
         <v>24</v>
       </c>
       <c r="H39" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I39" t="s">
         <v>29</v>
@@ -3264,21 +3265,21 @@
         <v>30</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B40" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C40" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D40" t="s">
         <v>21</v>
       </c>
       <c r="E40" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F40" t="s">
         <v>23</v>
@@ -3287,7 +3288,7 @@
         <v>24</v>
       </c>
       <c r="H40" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I40" t="s">
         <v>29</v>
@@ -3314,18 +3315,18 @@
         <v>29</v>
       </c>
       <c r="Q40" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="41" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B41" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C41" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D41" t="s">
         <v>21</v>
@@ -3340,7 +3341,7 @@
         <v>24</v>
       </c>
       <c r="H41" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I41" t="s">
         <v>29</v>
@@ -3370,21 +3371,21 @@
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B42" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C42" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D42" t="s">
         <v>21</v>
       </c>
       <c r="E42" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F42" t="s">
         <v>23</v>
@@ -3393,7 +3394,7 @@
         <v>24</v>
       </c>
       <c r="H42" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I42" t="s">
         <v>29</v>
@@ -3420,24 +3421,24 @@
         <v>29</v>
       </c>
       <c r="Q42" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="43" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B43" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C43" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D43" t="s">
         <v>21</v>
       </c>
       <c r="E43" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F43" t="s">
         <v>23</v>
@@ -3446,7 +3447,7 @@
         <v>24</v>
       </c>
       <c r="H43" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I43" t="s">
         <v>29</v>
@@ -3473,27 +3474,27 @@
         <v>29</v>
       </c>
       <c r="Q43" t="s">
+        <v>53</v>
+      </c>
+      <c r="R43" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>153</v>
+      </c>
+      <c r="B44" t="s">
+        <v>154</v>
+      </c>
+      <c r="C44" t="s">
         <v>49</v>
-      </c>
-      <c r="R43" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="44" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>157</v>
-      </c>
-      <c r="B44" t="s">
-        <v>158</v>
-      </c>
-      <c r="C44" t="s">
-        <v>45</v>
       </c>
       <c r="D44" t="s">
         <v>21</v>
       </c>
       <c r="E44" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F44" t="s">
         <v>23</v>
@@ -3502,7 +3503,7 @@
         <v>24</v>
       </c>
       <c r="H44" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I44" t="s">
         <v>29</v>
@@ -3529,21 +3530,21 @@
         <v>29</v>
       </c>
       <c r="Q44" t="s">
+        <v>53</v>
+      </c>
+      <c r="R44" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>155</v>
+      </c>
+      <c r="B45" t="s">
+        <v>156</v>
+      </c>
+      <c r="C45" t="s">
         <v>49</v>
-      </c>
-      <c r="R44" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="45" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>159</v>
-      </c>
-      <c r="B45" t="s">
-        <v>160</v>
-      </c>
-      <c r="C45" t="s">
-        <v>45</v>
       </c>
       <c r="D45" t="s">
         <v>21</v>
@@ -3558,7 +3559,7 @@
         <v>24</v>
       </c>
       <c r="H45" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I45" t="s">
         <v>29</v>
@@ -3588,15 +3589,15 @@
         <v>30</v>
       </c>
       <c r="R45" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="46" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B46" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C46" t="s">
         <v>20</v>
@@ -3605,7 +3606,7 @@
         <v>21</v>
       </c>
       <c r="E46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F46" t="s">
         <v>23</v>
@@ -3614,13 +3615,13 @@
         <v>24</v>
       </c>
       <c r="H46" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I46" t="s">
         <v>29</v>
       </c>
       <c r="J46" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="K46" t="s">
         <v>28</v>
@@ -3641,27 +3642,27 @@
         <v>29</v>
       </c>
       <c r="Q46" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="R46" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="47" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B47" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C47" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D47" t="s">
         <v>21</v>
       </c>
       <c r="E47" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F47" t="s">
         <v>23</v>
@@ -3670,13 +3671,13 @@
         <v>24</v>
       </c>
       <c r="H47" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I47" t="s">
         <v>29</v>
       </c>
       <c r="J47" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="K47" t="s">
         <v>28</v>
@@ -3691,21 +3692,21 @@
         <v>29</v>
       </c>
       <c r="O47" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P47" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Q47" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B48" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C48" t="s">
         <v>20</v>
@@ -3714,7 +3715,7 @@
         <v>21</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F48" t="s">
         <v>23</v>
@@ -3723,13 +3724,13 @@
         <v>24</v>
       </c>
       <c r="H48" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I48" t="s">
         <v>29</v>
       </c>
       <c r="J48" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="K48" t="s">
         <v>28</v>
@@ -3750,27 +3751,27 @@
         <v>29</v>
       </c>
       <c r="Q48" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="R48" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="49" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B49" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C49" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D49" t="s">
         <v>21</v>
       </c>
       <c r="E49" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F49" t="s">
         <v>23</v>
@@ -3779,7 +3780,7 @@
         <v>24</v>
       </c>
       <c r="H49" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I49" t="s">
         <v>29</v>
@@ -3806,27 +3807,27 @@
         <v>29</v>
       </c>
       <c r="Q49" t="s">
-        <v>85</v>
+        <v>172</v>
       </c>
       <c r="R49" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="50" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B50" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C50" t="s">
         <v>20</v>
       </c>
       <c r="D50" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E50" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F50" t="s">
         <v>23</v>
@@ -3835,13 +3836,13 @@
         <v>24</v>
       </c>
       <c r="H50" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I50" t="s">
         <v>29</v>
       </c>
       <c r="J50" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K50" t="s">
         <v>28</v>
@@ -3856,30 +3857,30 @@
         <v>29</v>
       </c>
       <c r="O50" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="P50" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="Q50" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B51" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C51" t="s">
         <v>20</v>
       </c>
       <c r="D51" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E51" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F51" t="s">
         <v>23</v>
@@ -3888,51 +3889,51 @@
         <v>24</v>
       </c>
       <c r="H51" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I51" t="s">
+        <v>179</v>
+      </c>
+      <c r="J51" t="s">
+        <v>27</v>
+      </c>
+      <c r="K51" t="s">
+        <v>28</v>
+      </c>
+      <c r="L51" t="s">
+        <v>28</v>
+      </c>
+      <c r="M51" t="s">
+        <v>29</v>
+      </c>
+      <c r="N51" t="s">
+        <v>29</v>
+      </c>
+      <c r="O51" t="s">
+        <v>84</v>
+      </c>
+      <c r="P51" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>181</v>
+      </c>
+      <c r="B52" t="s">
         <v>182</v>
       </c>
-      <c r="J51" t="s">
-        <v>61</v>
-      </c>
-      <c r="K51" t="s">
-        <v>28</v>
-      </c>
-      <c r="L51" t="s">
-        <v>28</v>
-      </c>
-      <c r="M51" t="s">
-        <v>29</v>
-      </c>
-      <c r="N51" t="s">
-        <v>29</v>
-      </c>
-      <c r="O51" t="s">
-        <v>88</v>
-      </c>
-      <c r="P51" t="s">
-        <v>183</v>
-      </c>
-      <c r="Q51" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="52" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>184</v>
-      </c>
-      <c r="B52" t="s">
-        <v>185</v>
-      </c>
       <c r="C52" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D52" t="s">
         <v>21</v>
       </c>
       <c r="E52" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F52" t="s">
         <v>23</v>
@@ -3941,13 +3942,13 @@
         <v>24</v>
       </c>
       <c r="H52" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I52" t="s">
         <v>29</v>
       </c>
       <c r="J52" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="K52" t="s">
         <v>28</v>
@@ -3968,24 +3969,24 @@
         <v>29</v>
       </c>
       <c r="Q52" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="53" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B53" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C53" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D53" t="s">
         <v>21</v>
       </c>
       <c r="E53" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F53" t="s">
         <v>23</v>
@@ -3994,13 +3995,13 @@
         <v>24</v>
       </c>
       <c r="H53" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I53" t="s">
         <v>29</v>
       </c>
       <c r="J53" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="K53" t="s">
         <v>28</v>
@@ -4021,98 +4022,98 @@
         <v>29</v>
       </c>
       <c r="Q53" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="R53" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="54" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B54" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C54" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D54" t="s">
         <v>21</v>
       </c>
       <c r="E54" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F54" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G54" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H54" t="s">
+        <v>189</v>
+      </c>
+      <c r="I54" t="s">
+        <v>29</v>
+      </c>
+      <c r="J54" t="s">
+        <v>29</v>
+      </c>
+      <c r="K54" t="s">
+        <v>28</v>
+      </c>
+      <c r="L54" t="s">
+        <v>28</v>
+      </c>
+      <c r="M54" t="s">
+        <v>29</v>
+      </c>
+      <c r="N54" t="s">
+        <v>29</v>
+      </c>
+      <c r="O54" t="s">
+        <v>29</v>
+      </c>
+      <c r="P54" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>53</v>
+      </c>
+      <c r="R54" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>191</v>
+      </c>
+      <c r="B55" t="s">
         <v>192</v>
       </c>
-      <c r="I54" t="s">
-        <v>29</v>
-      </c>
-      <c r="J54" t="s">
-        <v>29</v>
-      </c>
-      <c r="K54" t="s">
-        <v>28</v>
-      </c>
-      <c r="L54" t="s">
-        <v>28</v>
-      </c>
-      <c r="M54" t="s">
-        <v>29</v>
-      </c>
-      <c r="N54" t="s">
-        <v>29</v>
-      </c>
-      <c r="O54" t="s">
-        <v>29</v>
-      </c>
-      <c r="P54" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q54" t="s">
-        <v>49</v>
-      </c>
-      <c r="R54" t="s">
+      <c r="C55" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="55" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
+      <c r="D55" t="s">
         <v>194</v>
       </c>
-      <c r="B55" t="s">
+      <c r="E55" t="s">
+        <v>63</v>
+      </c>
+      <c r="F55" t="s">
+        <v>23</v>
+      </c>
+      <c r="G55" t="s">
+        <v>24</v>
+      </c>
+      <c r="H55" t="s">
         <v>195</v>
       </c>
-      <c r="C55" t="s">
-        <v>20</v>
-      </c>
-      <c r="D55" t="s">
-        <v>69</v>
-      </c>
-      <c r="E55" t="s">
-        <v>22</v>
-      </c>
-      <c r="F55" t="s">
-        <v>23</v>
-      </c>
-      <c r="G55" t="s">
-        <v>92</v>
-      </c>
-      <c r="H55" t="s">
-        <v>111</v>
-      </c>
       <c r="I55" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="J55" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="K55" t="s">
         <v>28</v>
@@ -4121,10 +4122,10 @@
         <v>28</v>
       </c>
       <c r="M55" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="N55" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="O55" t="s">
         <v>29</v>
@@ -4133,21 +4134,24 @@
         <v>29</v>
       </c>
       <c r="Q55" t="s">
-        <v>30</v>
+        <v>65</v>
+      </c>
+      <c r="R55" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="56" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B56" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C56" t="s">
         <v>20</v>
       </c>
       <c r="D56" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E56" t="s">
         <v>22</v>
@@ -4156,16 +4160,16 @@
         <v>23</v>
       </c>
       <c r="G56" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="H56" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="I56" t="s">
-        <v>182</v>
+        <v>80</v>
       </c>
       <c r="J56" t="s">
-        <v>198</v>
+        <v>40</v>
       </c>
       <c r="K56" t="s">
         <v>28</v>
@@ -4174,10 +4178,10 @@
         <v>28</v>
       </c>
       <c r="M56" t="s">
-        <v>70</v>
+        <v>195</v>
       </c>
       <c r="N56" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O56" t="s">
         <v>29</v>
@@ -4200,7 +4204,7 @@
         <v>20</v>
       </c>
       <c r="D57" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E57" t="s">
         <v>22</v>
@@ -4212,13 +4216,13 @@
         <v>24</v>
       </c>
       <c r="H57" t="s">
-        <v>83</v>
+        <v>118</v>
       </c>
       <c r="I57" t="s">
-        <v>29</v>
+        <v>179</v>
       </c>
       <c r="J57" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="K57" t="s">
         <v>28</v>
@@ -4227,10 +4231,10 @@
         <v>28</v>
       </c>
       <c r="M57" t="s">
-        <v>70</v>
+        <v>195</v>
       </c>
       <c r="N57" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O57" t="s">
         <v>29</v>
@@ -4244,19 +4248,19 @@
     </row>
     <row r="58" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B58" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C58" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="D58" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E58" t="s">
-        <v>103</v>
+        <v>22</v>
       </c>
       <c r="F58" t="s">
         <v>23</v>
@@ -4268,10 +4272,10 @@
         <v>79</v>
       </c>
       <c r="I58" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="J58" t="s">
-        <v>79</v>
+        <v>201</v>
       </c>
       <c r="K58" t="s">
         <v>28</v>
@@ -4280,10 +4284,10 @@
         <v>28</v>
       </c>
       <c r="M58" t="s">
-        <v>79</v>
+        <v>195</v>
       </c>
       <c r="N58" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="O58" t="s">
         <v>29</v>
@@ -4292,39 +4296,39 @@
         <v>29</v>
       </c>
       <c r="Q58" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="59" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B59" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C59" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
       <c r="D59" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E59" t="s">
-        <v>48</v>
+        <v>99</v>
       </c>
       <c r="F59" t="s">
-        <v>205</v>
+        <v>23</v>
       </c>
       <c r="G59" t="s">
         <v>24</v>
       </c>
       <c r="H59" t="s">
-        <v>122</v>
+        <v>75</v>
       </c>
       <c r="I59" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="J59" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="K59" t="s">
         <v>28</v>
@@ -4333,10 +4337,10 @@
         <v>28</v>
       </c>
       <c r="M59" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="N59" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="O59" t="s">
         <v>29</v>
@@ -4345,10 +4349,10 @@
         <v>29</v>
       </c>
       <c r="Q59" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="60" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>206</v>
       </c>
@@ -4356,28 +4360,28 @@
         <v>207</v>
       </c>
       <c r="C60" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
       <c r="D60" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E60" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F60" t="s">
-        <v>205</v>
+        <v>23</v>
       </c>
       <c r="G60" t="s">
         <v>24</v>
       </c>
       <c r="H60" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I60" t="s">
         <v>29</v>
       </c>
       <c r="J60" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="K60" t="s">
         <v>28</v>
@@ -4386,10 +4390,10 @@
         <v>28</v>
       </c>
       <c r="M60" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N60" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O60" t="s">
         <v>29</v>
@@ -4398,66 +4402,66 @@
         <v>29</v>
       </c>
       <c r="Q60" t="s">
-        <v>49</v>
-      </c>
-      <c r="R60" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="61" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
+      <c r="B61" t="s">
         <v>209</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
+        <v>193</v>
+      </c>
+      <c r="D61" t="s">
+        <v>194</v>
+      </c>
+      <c r="E61" t="s">
+        <v>52</v>
+      </c>
+      <c r="F61" t="s">
+        <v>23</v>
+      </c>
+      <c r="G61" t="s">
+        <v>24</v>
+      </c>
+      <c r="H61" t="s">
+        <v>118</v>
+      </c>
+      <c r="I61" t="s">
+        <v>29</v>
+      </c>
+      <c r="J61" t="s">
+        <v>79</v>
+      </c>
+      <c r="K61" t="s">
+        <v>28</v>
+      </c>
+      <c r="L61" t="s">
+        <v>28</v>
+      </c>
+      <c r="M61" t="s">
+        <v>79</v>
+      </c>
+      <c r="N61" t="s">
+        <v>88</v>
+      </c>
+      <c r="O61" t="s">
+        <v>29</v>
+      </c>
+      <c r="P61" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>53</v>
+      </c>
+      <c r="R61" t="s">
         <v>210</v>
       </c>
-      <c r="C61" t="s">
-        <v>68</v>
-      </c>
-      <c r="D61" t="s">
-        <v>69</v>
-      </c>
-      <c r="E61" t="s">
-        <v>22</v>
-      </c>
-      <c r="F61" t="s">
-        <v>23</v>
-      </c>
-      <c r="G61" t="s">
-        <v>24</v>
-      </c>
-      <c r="H61" t="s">
-        <v>122</v>
-      </c>
-      <c r="I61" t="s">
-        <v>29</v>
-      </c>
-      <c r="J61" t="s">
-        <v>83</v>
-      </c>
-      <c r="K61" t="s">
-        <v>28</v>
-      </c>
-      <c r="L61" t="s">
-        <v>28</v>
-      </c>
-      <c r="M61" t="s">
-        <v>83</v>
-      </c>
-      <c r="N61" t="s">
-        <v>92</v>
-      </c>
-      <c r="O61" t="s">
-        <v>29</v>
-      </c>
-      <c r="P61" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q61" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="62" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="62" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>211</v>
       </c>
@@ -4465,28 +4469,28 @@
         <v>212</v>
       </c>
       <c r="C62" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
       <c r="D62" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E62" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F62" t="s">
-        <v>205</v>
+        <v>23</v>
       </c>
       <c r="G62" t="s">
         <v>24</v>
       </c>
       <c r="H62" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I62" t="s">
         <v>29</v>
       </c>
       <c r="J62" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="K62" t="s">
         <v>28</v>
@@ -4495,10 +4499,10 @@
         <v>28</v>
       </c>
       <c r="M62" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N62" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O62" t="s">
         <v>29</v>
@@ -4507,122 +4511,122 @@
         <v>29</v>
       </c>
       <c r="Q62" t="s">
-        <v>49</v>
-      </c>
-      <c r="R62" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="63" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
+      <c r="B63" t="s">
         <v>214</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
+        <v>193</v>
+      </c>
+      <c r="D63" t="s">
+        <v>194</v>
+      </c>
+      <c r="E63" t="s">
+        <v>52</v>
+      </c>
+      <c r="F63" t="s">
+        <v>23</v>
+      </c>
+      <c r="G63" t="s">
+        <v>24</v>
+      </c>
+      <c r="H63" t="s">
+        <v>118</v>
+      </c>
+      <c r="I63" t="s">
+        <v>29</v>
+      </c>
+      <c r="J63" t="s">
+        <v>79</v>
+      </c>
+      <c r="K63" t="s">
+        <v>28</v>
+      </c>
+      <c r="L63" t="s">
+        <v>28</v>
+      </c>
+      <c r="M63" t="s">
+        <v>79</v>
+      </c>
+      <c r="N63" t="s">
+        <v>88</v>
+      </c>
+      <c r="O63" t="s">
+        <v>29</v>
+      </c>
+      <c r="P63" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>53</v>
+      </c>
+      <c r="R63" t="s">
         <v>215</v>
       </c>
-      <c r="C63" t="s">
-        <v>68</v>
-      </c>
-      <c r="D63" t="s">
-        <v>69</v>
-      </c>
-      <c r="E63" t="s">
-        <v>48</v>
-      </c>
-      <c r="F63" t="s">
-        <v>205</v>
-      </c>
-      <c r="G63" t="s">
-        <v>24</v>
-      </c>
-      <c r="H63" t="s">
-        <v>122</v>
-      </c>
-      <c r="I63" t="s">
-        <v>29</v>
-      </c>
-      <c r="J63" t="s">
-        <v>83</v>
-      </c>
-      <c r="K63" t="s">
-        <v>28</v>
-      </c>
-      <c r="L63" t="s">
-        <v>28</v>
-      </c>
-      <c r="M63" t="s">
-        <v>83</v>
-      </c>
-      <c r="N63" t="s">
-        <v>92</v>
-      </c>
-      <c r="O63" t="s">
-        <v>29</v>
-      </c>
-      <c r="P63" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q63" t="s">
-        <v>49</v>
-      </c>
-      <c r="R63" t="s">
+    </row>
+    <row r="64" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="64" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
+      <c r="B64" t="s">
         <v>217</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
+        <v>193</v>
+      </c>
+      <c r="D64" t="s">
+        <v>194</v>
+      </c>
+      <c r="E64" t="s">
+        <v>52</v>
+      </c>
+      <c r="F64" t="s">
+        <v>23</v>
+      </c>
+      <c r="G64" t="s">
+        <v>24</v>
+      </c>
+      <c r="H64" t="s">
+        <v>118</v>
+      </c>
+      <c r="I64" t="s">
+        <v>29</v>
+      </c>
+      <c r="J64" t="s">
+        <v>79</v>
+      </c>
+      <c r="K64" t="s">
+        <v>28</v>
+      </c>
+      <c r="L64" t="s">
+        <v>28</v>
+      </c>
+      <c r="M64" t="s">
+        <v>79</v>
+      </c>
+      <c r="N64" t="s">
+        <v>88</v>
+      </c>
+      <c r="O64" t="s">
+        <v>29</v>
+      </c>
+      <c r="P64" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>53</v>
+      </c>
+      <c r="R64" t="s">
         <v>218</v>
       </c>
-      <c r="C64" t="s">
-        <v>68</v>
-      </c>
-      <c r="D64" t="s">
-        <v>69</v>
-      </c>
-      <c r="E64" t="s">
-        <v>22</v>
-      </c>
-      <c r="F64" t="s">
-        <v>23</v>
-      </c>
-      <c r="G64" t="s">
-        <v>24</v>
-      </c>
-      <c r="H64" t="s">
-        <v>122</v>
-      </c>
-      <c r="I64" t="s">
-        <v>29</v>
-      </c>
-      <c r="J64" t="s">
-        <v>83</v>
-      </c>
-      <c r="K64" t="s">
-        <v>28</v>
-      </c>
-      <c r="L64" t="s">
-        <v>28</v>
-      </c>
-      <c r="M64" t="s">
-        <v>83</v>
-      </c>
-      <c r="N64" t="s">
-        <v>92</v>
-      </c>
-      <c r="O64" t="s">
-        <v>29</v>
-      </c>
-      <c r="P64" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q64" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="65" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="65" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>219</v>
       </c>
@@ -4630,10 +4634,10 @@
         <v>220</v>
       </c>
       <c r="C65" t="s">
-        <v>20</v>
+        <v>193</v>
       </c>
       <c r="D65" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E65" t="s">
         <v>22</v>
@@ -4645,13 +4649,13 @@
         <v>24</v>
       </c>
       <c r="H65" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I65" t="s">
         <v>29</v>
       </c>
       <c r="J65" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="K65" t="s">
         <v>28</v>
@@ -4660,10 +4664,10 @@
         <v>28</v>
       </c>
       <c r="M65" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N65" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O65" t="s">
         <v>29</v>
@@ -4686,10 +4690,10 @@
         <v>20</v>
       </c>
       <c r="D66" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E66" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="F66" t="s">
         <v>23</v>
@@ -4698,13 +4702,13 @@
         <v>24</v>
       </c>
       <c r="H66" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
       <c r="I66" t="s">
         <v>29</v>
       </c>
       <c r="J66" t="s">
-        <v>29</v>
+        <v>107</v>
       </c>
       <c r="K66" t="s">
         <v>28</v>
@@ -4713,10 +4717,10 @@
         <v>28</v>
       </c>
       <c r="M66" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N66" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O66" t="s">
         <v>29</v>
@@ -4725,27 +4729,24 @@
         <v>29</v>
       </c>
       <c r="Q66" t="s">
-        <v>62</v>
-      </c>
-      <c r="R66" t="s">
-        <v>223</v>
+        <v>30</v>
       </c>
     </row>
     <row r="67" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
+        <v>223</v>
+      </c>
+      <c r="B67" t="s">
         <v>224</v>
-      </c>
-      <c r="B67" t="s">
-        <v>225</v>
       </c>
       <c r="C67" t="s">
         <v>20</v>
       </c>
       <c r="D67" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E67" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F67" t="s">
         <v>23</v>
@@ -4754,7 +4755,7 @@
         <v>24</v>
       </c>
       <c r="H67" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="I67" t="s">
         <v>29</v>
@@ -4769,10 +4770,10 @@
         <v>28</v>
       </c>
       <c r="M67" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N67" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O67" t="s">
         <v>29</v>
@@ -4781,7 +4782,10 @@
         <v>29</v>
       </c>
       <c r="Q67" t="s">
-        <v>62</v>
+        <v>65</v>
+      </c>
+      <c r="R67" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="68" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
@@ -4795,10 +4799,10 @@
         <v>20</v>
       </c>
       <c r="D68" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E68" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="F68" t="s">
         <v>23</v>
@@ -4807,13 +4811,13 @@
         <v>24</v>
       </c>
       <c r="H68" t="s">
-        <v>228</v>
+        <v>92</v>
       </c>
       <c r="I68" t="s">
-        <v>228</v>
+        <v>29</v>
       </c>
       <c r="J68" t="s">
-        <v>229</v>
+        <v>29</v>
       </c>
       <c r="K68" t="s">
         <v>28</v>
@@ -4822,10 +4826,10 @@
         <v>28</v>
       </c>
       <c r="M68" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N68" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O68" t="s">
         <v>29</v>
@@ -4834,24 +4838,24 @@
         <v>29</v>
       </c>
       <c r="Q68" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
     </row>
     <row r="69" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B69" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C69" t="s">
         <v>20</v>
       </c>
       <c r="D69" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E69" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="F69" t="s">
         <v>23</v>
@@ -4860,13 +4864,13 @@
         <v>24</v>
       </c>
       <c r="H69" t="s">
-        <v>122</v>
+        <v>230</v>
       </c>
       <c r="I69" t="s">
-        <v>29</v>
+        <v>230</v>
       </c>
       <c r="J69" t="s">
-        <v>111</v>
+        <v>231</v>
       </c>
       <c r="K69" t="s">
         <v>28</v>
@@ -4875,10 +4879,10 @@
         <v>28</v>
       </c>
       <c r="M69" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N69" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O69" t="s">
         <v>29</v>
@@ -4887,7 +4891,7 @@
         <v>29</v>
       </c>
       <c r="Q69" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
     </row>
     <row r="70" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
@@ -4898,28 +4902,28 @@
         <v>233</v>
       </c>
       <c r="C70" t="s">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="D70" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E70" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F70" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G70" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="H70" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I70" t="s">
         <v>29</v>
       </c>
       <c r="J70" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="K70" t="s">
         <v>28</v>
@@ -4928,10 +4932,10 @@
         <v>28</v>
       </c>
       <c r="M70" t="s">
-        <v>122</v>
+        <v>79</v>
       </c>
       <c r="N70" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="O70" t="s">
         <v>29</v>
@@ -4943,7 +4947,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>234</v>
       </c>
@@ -4951,81 +4955,81 @@
         <v>235</v>
       </c>
       <c r="C71" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
       <c r="D71" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E71" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F71" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="G71" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H71" t="s">
+        <v>118</v>
+      </c>
+      <c r="I71" t="s">
+        <v>29</v>
+      </c>
+      <c r="J71" t="s">
+        <v>118</v>
+      </c>
+      <c r="K71" t="s">
+        <v>28</v>
+      </c>
+      <c r="L71" t="s">
+        <v>28</v>
+      </c>
+      <c r="M71" t="s">
+        <v>118</v>
+      </c>
+      <c r="N71" t="s">
+        <v>24</v>
+      </c>
+      <c r="O71" t="s">
+        <v>29</v>
+      </c>
+      <c r="P71" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="72" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
         <v>236</v>
       </c>
-      <c r="I71" t="s">
-        <v>29</v>
-      </c>
-      <c r="J71" t="s">
-        <v>192</v>
-      </c>
-      <c r="K71" t="s">
-        <v>28</v>
-      </c>
-      <c r="L71" t="s">
-        <v>28</v>
-      </c>
-      <c r="M71" t="s">
-        <v>192</v>
-      </c>
-      <c r="N71" t="s">
-        <v>92</v>
-      </c>
-      <c r="O71" t="s">
-        <v>29</v>
-      </c>
-      <c r="P71" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q71" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="72" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
+      <c r="B72" t="s">
         <v>237</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
+        <v>193</v>
+      </c>
+      <c r="D72" t="s">
+        <v>194</v>
+      </c>
+      <c r="E72" t="s">
+        <v>99</v>
+      </c>
+      <c r="F72" t="s">
+        <v>88</v>
+      </c>
+      <c r="G72" t="s">
+        <v>88</v>
+      </c>
+      <c r="H72" t="s">
         <v>238</v>
       </c>
-      <c r="C72" t="s">
-        <v>68</v>
-      </c>
-      <c r="D72" t="s">
-        <v>69</v>
-      </c>
-      <c r="E72" t="s">
-        <v>48</v>
-      </c>
-      <c r="F72" t="s">
-        <v>92</v>
-      </c>
-      <c r="G72" t="s">
-        <v>92</v>
-      </c>
-      <c r="H72" t="s">
-        <v>192</v>
-      </c>
       <c r="I72" t="s">
         <v>29</v>
       </c>
       <c r="J72" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="K72" t="s">
         <v>28</v>
@@ -5034,10 +5038,10 @@
         <v>28</v>
       </c>
       <c r="M72" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="N72" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O72" t="s">
         <v>29</v>
@@ -5046,10 +5050,10 @@
         <v>29</v>
       </c>
       <c r="Q72" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="73" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="73" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>239</v>
       </c>
@@ -5057,28 +5061,28 @@
         <v>240</v>
       </c>
       <c r="C73" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
       <c r="D73" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E73" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F73" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G73" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H73" t="s">
-        <v>236</v>
+        <v>189</v>
       </c>
       <c r="I73" t="s">
         <v>29</v>
       </c>
       <c r="J73" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="K73" t="s">
         <v>28</v>
@@ -5087,10 +5091,10 @@
         <v>28</v>
       </c>
       <c r="M73" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="N73" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O73" t="s">
         <v>29</v>
@@ -5099,10 +5103,10 @@
         <v>29</v>
       </c>
       <c r="Q73" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="74" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="74" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>241</v>
       </c>
@@ -5110,28 +5114,28 @@
         <v>242</v>
       </c>
       <c r="C74" t="s">
-        <v>68</v>
+        <v>193</v>
       </c>
       <c r="D74" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
       <c r="E74" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F74" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G74" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H74" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="I74" t="s">
         <v>29</v>
       </c>
       <c r="J74" t="s">
-        <v>236</v>
+        <v>189</v>
       </c>
       <c r="K74" t="s">
         <v>28</v>
@@ -5140,10 +5144,10 @@
         <v>28</v>
       </c>
       <c r="M74" t="s">
-        <v>236</v>
+        <v>189</v>
       </c>
       <c r="N74" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O74" t="s">
         <v>29</v>
@@ -5152,10 +5156,10 @@
         <v>29</v>
       </c>
       <c r="Q74" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="75" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="75" spans="1:18" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>243</v>
       </c>
@@ -5163,28 +5167,28 @@
         <v>244</v>
       </c>
       <c r="C75" t="s">
-        <v>20</v>
+        <v>193</v>
       </c>
       <c r="D75" t="s">
-        <v>21</v>
+        <v>194</v>
       </c>
       <c r="E75" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="F75" t="s">
-        <v>23</v>
+        <v>88</v>
       </c>
       <c r="G75" t="s">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="H75" t="s">
-        <v>71</v>
+        <v>238</v>
       </c>
       <c r="I75" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="J75" t="s">
-        <v>61</v>
+        <v>238</v>
       </c>
       <c r="K75" t="s">
         <v>28</v>
@@ -5193,10 +5197,10 @@
         <v>28</v>
       </c>
       <c r="M75" t="s">
-        <v>29</v>
+        <v>238</v>
       </c>
       <c r="N75" t="s">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="O75" t="s">
         <v>29</v>
@@ -5205,13 +5209,20 @@
         <v>29</v>
       </c>
       <c r="Q75" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="C1:C75" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Execução"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:R48 A73:R75 A72:P72 R72 A71:P71 R71 A50:R70 A49:P49 R49" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:R75" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5246,7 +5257,7 @@
         <v>249</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>